<commit_message>
Fix: building 'criar_planilha.py' and adding '.env.example'
</commit_message>
<xml_diff>
--- a/funcionarios.xlsx
+++ b/funcionarios.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contatos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,26 +25,13 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -59,12 +46,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -456,136 +442,136 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Ana Souza</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>ana.souza@example.com</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Vendas</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Bruno Lima</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>bruno.lima@example.com</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Carla Mendes</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>carla.mendes@example.com</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Financeiro</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Diego Alves</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>diego.alves@example.com</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Vendas</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Eduarda Rocha</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>eduarda.rocha@example.com</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Logística</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Felipe Costa</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>felipe.costa@example.com</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Gabriela Nunes</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>gabriela.nunes@example.com</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Financeiro</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Henrique Dias</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>henrique.dias@example.com</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Diretoria</t>
         </is>

</xml_diff>

<commit_message>
Feature: saving sent email registers at funcionarios.xlsx
</commit_message>
<xml_diff>
--- a/funcionarios.xlsx
+++ b/funcionarios.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Registros" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -580,4 +581,216 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Nome</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ana Souza</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ana.souza@example.com</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>07/10/2026 23:49:05</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Enviado com sucesso</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Bruno Lima</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>bruno.lima@example.com</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>07/10/2026 23:49:14</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Enviado com sucesso</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Carla Mendes</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>carla.mendes@example.com</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>07/10/2026 23:49:23</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Enviado com sucesso</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Diego Alves</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>diego.alves@example.com</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>07/10/2026 23:49:32</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Enviado com sucesso</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Eduarda Rocha</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>eduarda.rocha@example.com</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>07/10/2026 23:49:41</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Enviado com sucesso</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Felipe Costa</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>felipe.costa@example.com</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>07/10/2026 23:49:50</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Enviado com sucesso</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Gabriela Nunes</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>gabriela.nunes@example.com</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>07/10/2026 23:49:59</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Enviado com sucesso</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Henrique Dias</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>henrique.dias@example.com</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>07/10/2026 23:50:08</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Enviado com sucesso</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Feature: selecting and registering type of sent
</commit_message>
<xml_diff>
--- a/funcionarios.xlsx
+++ b/funcionarios.xlsx
@@ -2,29 +2,34 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Registros" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="2">
@@ -35,7 +40,14 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left/>
       <right/>
@@ -45,16 +57,18 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -203,6 +217,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -237,6 +252,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -260,7 +276,6 @@
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
                 <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
@@ -271,31 +286,31 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
+                <a:tint val="51000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="80000">
               <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
+                <a:tint val="15000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
+                <a:tint val="94000"/>
                 <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
         <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
+              <a:shade val="9500"/>
               <a:satMod val="105000"/>
             </a:schemeClr>
           </a:solidFill>
@@ -317,7 +332,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -375,7 +390,7 @@
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
+                <a:tint val="20000"/>
                 <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
@@ -388,13 +403,12 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
                 <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
                 <a:satMod val="200000"/>
               </a:schemeClr>
             </a:gs>
@@ -414,35 +428,35 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="22" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
+    <col width="34" bestFit="1" customWidth="1" style="2" min="2" max="2"/>
+    <col width="16" bestFit="1" customWidth="1" style="2" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="18.75" customHeight="1" s="2">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Nome</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Setor</t>
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="18.75" customHeight="1" s="2">
       <c r="A2" t="inlineStr">
         <is>
           <t>Ana Souza</t>
@@ -459,7 +473,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="18.75" customHeight="1" s="2">
       <c r="A3" t="inlineStr">
         <is>
           <t>Bruno Lima</t>
@@ -476,7 +490,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="18.75" customHeight="1" s="2">
       <c r="A4" t="inlineStr">
         <is>
           <t>Carla Mendes</t>
@@ -493,7 +507,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="18.75" customHeight="1" s="2">
       <c r="A5" t="inlineStr">
         <is>
           <t>Diego Alves</t>
@@ -510,7 +524,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="18.75" customHeight="1" s="2">
       <c r="A6" t="inlineStr">
         <is>
           <t>Eduarda Rocha</t>
@@ -527,7 +541,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="18.75" customHeight="1" s="2">
       <c r="A7" t="inlineStr">
         <is>
           <t>Felipe Costa</t>
@@ -544,7 +558,7 @@
         </is>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="18.75" customHeight="1" s="2">
       <c r="A8" t="inlineStr">
         <is>
           <t>Gabriela Nunes</t>
@@ -561,7 +575,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="18.75" customHeight="1" s="2">
       <c r="A9" t="inlineStr">
         <is>
           <t>Henrique Dias</t>
@@ -579,7 +593,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -589,7 +603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -605,10 +619,15 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>Tipo de envio</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>Data</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -617,174 +636,25 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Ana Souza</t>
+          <t>Henrique Dias</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ana.souza@example.com</t>
+          <t>henrique.dias@example.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>07/10/2026 23:49:05</t>
+          <t>Diretoria</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Enviado com sucesso</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Bruno Lima</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>bruno.lima@example.com</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>07/10/2026 23:49:14</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Enviado com sucesso</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Carla Mendes</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>carla.mendes@example.com</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>07/10/2026 23:49:23</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Enviado com sucesso</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Diego Alves</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>diego.alves@example.com</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>07/10/2026 23:49:32</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Enviado com sucesso</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Eduarda Rocha</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>eduarda.rocha@example.com</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>07/10/2026 23:49:41</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Enviado com sucesso</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Felipe Costa</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>felipe.costa@example.com</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>07/10/2026 23:49:50</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Enviado com sucesso</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Gabriela Nunes</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>gabriela.nunes@example.com</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>07/10/2026 23:49:59</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Enviado com sucesso</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Henrique Dias</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>henrique.dias@example.com</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>07/10/2026 23:50:08</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
+          <t>08/10/2026 00:40:34</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
         <is>
           <t>Enviado com sucesso</t>
         </is>

</xml_diff>